<commit_message>
Excersise Bai20 + Bai21 (#8)
* upload bai17

* upload bai18

* upadate file pom

* Upload Smoke Test xml

* upload bai 19

* upload bai 19

* temporaly save

* resolve conflict changes

* update bai20

* Delete src/test/java/com/Bai19/Bai19_LoginTestDDT.java

* Delete src/test/java/com/Bai20/Bai20.java

* Delete pom.xml

* Delete src/test/resources/suites/Test1.xml

* Revert "Delete pom.xml"

This reverts commit 755493800f26e9433d676952456d30a4bf88adac.

* Upload Exercise: Bai-21

* remove thread sleep

* update pom

* upload excesice Bonus Upload File

* Update bonus excersise for upload-file and drag-and-drop

* update test DragAndDrop

* resolve comments
</commit_message>
<xml_diff>
--- a/src/test/resources/data/TestDataBai19.xlsx
+++ b/src/test/resources/data/TestDataBai19.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="27">
   <si>
     <t>TestcaseID</t>
   </si>
@@ -447,13 +447,13 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="3" width="9.719285714285713" collapsed="false"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="3" width="33.43357142857143" collapsed="false"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="3" width="26.862142857142857" collapsed="false"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="3" width="18.14785714285714" collapsed="false"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="3" width="24.576428571428572" collapsed="false"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="3" width="11.147857142857141" collapsed="false"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="3" width="9.862142857142858" collapsed="false"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="3" width="9.719285714285713" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="3" width="33.43357142857143" collapsed="true"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="3" width="26.862142857142857" collapsed="true"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="3" width="18.14785714285714" collapsed="true"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="3" width="24.576428571428572" collapsed="true"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="3" width="11.147857142857141" collapsed="true"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="3" width="9.862142857142858" collapsed="true"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">

</xml_diff>